<commit_message>
Create copy of US develop branch
</commit_message>
<xml_diff>
--- a/InputData/bldgs/EoBSDwEC/Elast of Bldg Svc Demand wrt E Cost.xlsx
+++ b/InputData/bldgs/EoBSDwEC/Elast of Bldg Svc Demand wrt E Cost.xlsx
@@ -1,35 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="21929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="26227"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\deept\Dropbox\EPS\Input Data for India 2.0\bldgs\EoBSDwEC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rachel Goldstein\Dropbox (Energy Innovation)\Desktop\Vensim files from GitHub\EPS US\InputData\bldgs\EoBSDwEC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E50E48A-5001-4B0D-BE7C-1ACD0D3516B4}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="44" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{344434C8-6702-4CA8-9A05-280406723E48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30960" yWindow="2205" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
-    <sheet name="EoBSDwEC" sheetId="2" r:id="rId2"/>
+    <sheet name="AEO Assumptions" sheetId="3" r:id="rId2"/>
+    <sheet name="EoBSDwEC" sheetId="2" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="145621"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="32">
   <si>
     <t>EoBSDwEC Elasticity of Building Service Demand wrt Energy Cost</t>
   </si>
@@ -43,15 +36,9 @@
     <t>Residential</t>
   </si>
   <si>
-    <t>http://www.eia.gov/forecasts/aeo/assumptions/pdf/residential.pdf</t>
-  </si>
-  <si>
     <t>Commercial</t>
   </si>
   <si>
-    <t>http://www.eia.gov/forecasts/aeo/assumptions/pdf/commercial.pdf</t>
-  </si>
-  <si>
     <t>Notes:</t>
   </si>
   <si>
@@ -94,67 +81,43 @@
     <t>Rural Residential</t>
   </si>
   <si>
-    <t>Assumptions to the Annual Energy Outlook 2015</t>
-  </si>
-  <si>
-    <t>Residential Demand Module, Page 29</t>
-  </si>
-  <si>
-    <t>Commercial Demand Module, Page 42</t>
-  </si>
-  <si>
     <t>biomass</t>
   </si>
   <si>
+    <t>kerosene</t>
+  </si>
+  <si>
+    <t>heavy or residual fuel oil</t>
+  </si>
+  <si>
+    <t>LPG propane or butane</t>
+  </si>
+  <si>
+    <t>hydrogen</t>
+  </si>
+  <si>
     <t>Elasticity by Fuel (dimensionless)</t>
   </si>
   <si>
-    <t>kerosene</t>
-  </si>
-  <si>
-    <t>heavy or residual fuel oil</t>
-  </si>
-  <si>
-    <t>LPG propane or butane</t>
-  </si>
-  <si>
-    <t>hydrogen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The high elasticities in developing countries where consumption is constrained by distribution </t>
-  </si>
-  <si>
-    <t xml:space="preserve">US values are retained. </t>
-  </si>
-  <si>
-    <t>The review of India-specific studies is listed as a source for reference.</t>
-  </si>
-  <si>
-    <t>Review of Key International Demand Elasticities for Major Industrializing Economies</t>
-  </si>
-  <si>
-    <t>Energy Modeling Forum, Stanford University</t>
-  </si>
-  <si>
-    <t>Huntington et. al</t>
-  </si>
-  <si>
-    <t>https://web.stanford.edu/group/emf-research/docs/special_reports/EMF_SR12.pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">and other systemic factors (such as price distortions due to subsidies) could indicate </t>
-  </si>
-  <si>
-    <t>Hence the India-specific elasticities are not considered within this variable and</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(of the order of -0.41 (diesel), -0.65 (electricity) and -1.25 (natural gas)). </t>
-  </si>
-  <si>
-    <t xml:space="preserve">A few estimates are available for fuels in India. However, they indicate a high price elasticity  </t>
-  </si>
-  <si>
-    <t xml:space="preserve">changes in policy to expand infrastructure/access, rather than change in end-user behaviour. </t>
+    <t>Residential Demand Module</t>
+  </si>
+  <si>
+    <t>Commercial Demand Module</t>
+  </si>
+  <si>
+    <t>https://www.eia.gov/outlooks/aeo/assumptions/pdf/CDM_Assumptions.pdf</t>
+  </si>
+  <si>
+    <t>https://www.eia.gov/outlooks/aeo/assumptions/pdf/rDM_Assumptions.pdf</t>
+  </si>
+  <si>
+    <t>Assumptions to the Annual Energy Outlook 2023</t>
+  </si>
+  <si>
+    <t>Residential Demand Module, Page 10</t>
+  </si>
+  <si>
+    <t>Commercial Demand Module, Page 12</t>
   </si>
 </sst>
 </file>
@@ -186,18 +149,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.249977111117893"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -226,7 +183,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -243,6 +200,111 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>600925</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>67057</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Picture 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BD44B5EF-D9AC-FE06-7866-DB89594A951B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="4191000"/>
+          <a:ext cx="6087325" cy="2734057"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>600925</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>47951</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="Picture 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B0A2935C-7788-A00C-0A39-E609CA2C7CC6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="571500"/>
+          <a:ext cx="6087325" cy="2333951"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -566,175 +628,145 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K32"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="65" customWidth="1"/>
-    <col min="11" max="11" width="10.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="E3" s="6"/>
-      <c r="F3" s="6"/>
-      <c r="G3" s="6"/>
-      <c r="H3" s="6"/>
-      <c r="I3" s="6"/>
-      <c r="J3" s="6"/>
-      <c r="K3" s="6"/>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B4" s="2">
-        <v>2015</v>
-      </c>
-      <c r="D4" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
-        <v>21</v>
-      </c>
-      <c r="D5" s="2">
-        <v>2017</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="D6" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B7" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D7" s="3" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B8" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B11" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B9" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B11" s="1" t="s">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B13" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B12" s="3" t="s">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
         <v>6</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B13" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>32</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="D7" r:id="rId1" xr:uid="{8EC35FCC-D083-49D1-A161-BB9ACB23D295}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId2"/>
+  <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B545A04D-0C81-4573-BDE4-77F74558811D}">
+  <dimension ref="A1:I21"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>28</v>
+      </c>
+      <c r="I1" s="6">
+        <v>44986</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>27</v>
+      </c>
+      <c r="I20" s="6">
+        <v>44986</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <tabColor theme="3"/>
@@ -742,28 +774,28 @@
   <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24" customWidth="1"/>
+    <col min="1" max="1" width="25" customWidth="1"/>
     <col min="2" max="3" width="19.85546875" customWidth="1"/>
     <col min="4" max="4" width="14.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B2">
         <v>-0.3</v>
@@ -777,7 +809,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B3">
         <v>-0.15</v>
@@ -791,7 +823,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B4">
         <v>-0.15</v>
@@ -805,7 +837,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B5">
         <v>-0.15</v>
@@ -819,7 +851,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B6">
         <v>-0.15</v>
@@ -833,7 +865,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="B7">
         <v>-0.15</v>
@@ -847,7 +879,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="B8">
         <v>-0.15</v>
@@ -861,7 +893,7 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="B9">
         <v>-0.15</v>
@@ -875,7 +907,7 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="B10">
         <v>-0.15</v>
@@ -889,7 +921,7 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="B11">
         <v>-0.15</v>

</xml_diff>

<commit_message>
Files provided by WRI, with bug fixes
</commit_message>
<xml_diff>
--- a/InputData/bldgs/EoBSDwEC/Elast of Bldg Svc Demand wrt E Cost.xlsx
+++ b/InputData/bldgs/EoBSDwEC/Elast of Bldg Svc Demand wrt E Cost.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="26227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27706"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -17,7 +17,23 @@
     <sheet name="AEO Assumptions" sheetId="3" r:id="rId2"/>
     <sheet name="EoBSDwEC" sheetId="2" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="145621"/>
+  <calcPr calcId="191028"/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -33,12 +49,27 @@
     <t>U.S. Energy Information Administration</t>
   </si>
   <si>
+    <t>Assumptions to the Annual Energy Outlook 2023</t>
+  </si>
+  <si>
     <t>Residential</t>
   </si>
   <si>
+    <t>https://www.eia.gov/outlooks/aeo/assumptions/pdf/rDM_Assumptions.pdf</t>
+  </si>
+  <si>
+    <t>Residential Demand Module, Page 10</t>
+  </si>
+  <si>
     <t>Commercial</t>
   </si>
   <si>
+    <t>https://www.eia.gov/outlooks/aeo/assumptions/pdf/CDM_Assumptions.pdf</t>
+  </si>
+  <si>
+    <t>Commercial Demand Module, Page 12</t>
+  </si>
+  <si>
     <t>Notes:</t>
   </si>
   <si>
@@ -48,6 +79,33 @@
     <t>rather than equipment change in the model.</t>
   </si>
   <si>
+    <t>In the EIA source material, Residential elasticities are disaggregated by fuel,</t>
+  </si>
+  <si>
+    <t>while Commercial elasticities are not.  On the Commercial side, refrigeration</t>
+  </si>
+  <si>
+    <t>has a lower elasticity than other energy uses (-.1 instead of -.25), but we group</t>
+  </si>
+  <si>
+    <t>refrigeration with other appliances in our model and so disregard this difference.</t>
+  </si>
+  <si>
+    <t>Residential Demand Module</t>
+  </si>
+  <si>
+    <t>Commercial Demand Module</t>
+  </si>
+  <si>
+    <t>Elasticity by Fuel (dimensionless)</t>
+  </si>
+  <si>
+    <t>Urban Residential</t>
+  </si>
+  <si>
+    <t>Rural Residential</t>
+  </si>
+  <si>
     <t>electricity</t>
   </si>
   <si>
@@ -63,24 +121,6 @@
     <t>heat</t>
   </si>
   <si>
-    <t>In the EIA source material, Residential elasticities are disaggregated by fuel,</t>
-  </si>
-  <si>
-    <t>while Commercial elasticities are not.  On the Commercial side, refrigeration</t>
-  </si>
-  <si>
-    <t>has a lower elasticity than other energy uses (-.1 instead of -.25), but we group</t>
-  </si>
-  <si>
-    <t>refrigeration with other appliances in our model and so disregard this difference.</t>
-  </si>
-  <si>
-    <t>Urban Residential</t>
-  </si>
-  <si>
-    <t>Rural Residential</t>
-  </si>
-  <si>
     <t>biomass</t>
   </si>
   <si>
@@ -94,37 +134,13 @@
   </si>
   <si>
     <t>hydrogen</t>
-  </si>
-  <si>
-    <t>Elasticity by Fuel (dimensionless)</t>
-  </si>
-  <si>
-    <t>Residential Demand Module</t>
-  </si>
-  <si>
-    <t>Commercial Demand Module</t>
-  </si>
-  <si>
-    <t>https://www.eia.gov/outlooks/aeo/assumptions/pdf/CDM_Assumptions.pdf</t>
-  </si>
-  <si>
-    <t>https://www.eia.gov/outlooks/aeo/assumptions/pdf/rDM_Assumptions.pdf</t>
-  </si>
-  <si>
-    <t>Assumptions to the Annual Energy Outlook 2023</t>
-  </si>
-  <si>
-    <t>Residential Demand Module, Page 10</t>
-  </si>
-  <si>
-    <t>Commercial Demand Module, Page 12</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -308,9 +324,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -348,9 +364,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -383,26 +399,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -435,26 +434,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -629,17 +611,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B22"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="65" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -647,77 +629,77 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2">
       <c r="B4" s="2">
         <v>2023</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2">
       <c r="B5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
       <c r="B7" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
       <c r="B8" s="3" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
       <c r="B9" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
       <c r="B11" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
       <c r="B12" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
       <c r="B13" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2">
       <c r="A15" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2">
       <c r="A16" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1">
       <c r="A17" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1">
       <c r="A19" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:1">
       <c r="A20" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:1">
       <c r="A21" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:1">
       <c r="A22" t="s">
         <v>16</v>
       </c>
@@ -731,32 +713,32 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B545A04D-0C81-4573-BDE4-77F74558811D}">
   <dimension ref="A1:I21"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9">
       <c r="A1" t="s">
-        <v>28</v>
+        <v>5</v>
       </c>
       <c r="I1" s="6">
         <v>44986</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9">
       <c r="A2" s="1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9">
       <c r="A20" t="s">
-        <v>27</v>
+        <v>8</v>
       </c>
       <c r="I20" s="6">
         <v>44986</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9">
       <c r="A21" s="1" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -772,30 +754,30 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:D11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
     <col min="2" max="3" width="19.85546875" customWidth="1"/>
     <col min="4" max="4" width="14.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" ht="30">
       <c r="A1" s="5" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="B2">
         <v>-0.3</v>
@@ -807,9 +789,9 @@
         <v>-0.25</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="B3">
         <v>-0.15</v>
@@ -821,9 +803,9 @@
         <v>-0.25</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="B4">
         <v>-0.15</v>
@@ -835,9 +817,9 @@
         <v>-0.25</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="B5">
         <v>-0.15</v>
@@ -849,9 +831,9 @@
         <v>-0.25</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="B6">
         <v>-0.15</v>
@@ -863,9 +845,9 @@
         <v>-0.25</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="B7">
         <v>-0.15</v>
@@ -877,9 +859,9 @@
         <v>-0.25</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="B8">
         <v>-0.15</v>
@@ -891,9 +873,9 @@
         <v>-0.25</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="B9">
         <v>-0.15</v>
@@ -905,9 +887,9 @@
         <v>-0.25</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="B10">
         <v>-0.15</v>
@@ -919,9 +901,9 @@
         <v>-0.25</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="B11">
         <v>-0.15</v>
@@ -936,4 +918,175 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A251C7805F896F47A4F48569C73A0799" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="77cd1fc208aa16a525090c2a27f33c66">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f3083de3-5d4e-49f2-a3cd-0aeb079e6739" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d77402130d0e9b5bbfbb66ed18db98d9" ns2:_="">
+    <xsd:import namespace="f3083de3-5d4e-49f2-a3cd-0aeb079e6739"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="f3083de3-5d4e-49f2-a3cd-0aeb079e6739" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="10" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="11" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{83A8AE64-76C9-413B-8557-6197E4A1FE38}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0D27540F-D8AE-4B90-AF66-7A0DBDE855EC}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{13946EDF-0639-49AC-8DD9-D4A548E3C925}"/>
 </file>
</xml_diff>